<commit_message>
feat: implement error recovery, failure classification, and network tracking to improve Playwright test resilience
</commit_message>
<xml_diff>
--- a/input/UC_trail_pw.xlsx
+++ b/input/UC_trail_pw.xlsx
@@ -481,7 +481,7 @@
         <v>['Full Name: Text (max 50 chars, alphabets and spaces only)', 'Email Address: Text (max 100 chars, must be unique and valid format)', 'Role: Dropdown (must exist in Role Management)']</v>
       </c>
       <c r="I2" t="str">
-        <v>1. Navigate to User Management; 2. Click on Add User.; 3. click New Internal User.; 4. Enter first Name.; 5. Enter last Name.; 6. Enter Email Address.; 7. open the dropdown.; 8. Select Role.; 9. Click on Save.;</v>
+        <v>1. Navigate to User Management; 2. Click on Add User.; 3. click Add Internal User.; 4. Enter first Name.; 5. Enter last Name.; 6. Enter Email Address.; 7. open the role dropdown.; 8. Select Role.; 9. Click on Save.;</v>
       </c>
       <c r="J2" t="str">
         <v>1. User Management page is displayed.; 2. Add User form is displayed.; 3. Full Name field shows the entered value.; 4. Email Address field shows the entered value.; 5. Role dropdown reflects the chosen role.; 6. User is visible in the list with correct status with status Pending.; Overall: New user is listed in User Management with Pending status.</v>
@@ -649,7 +649,7 @@
         <v>['Email Address: Text (must not match any existing records)']</v>
       </c>
       <c r="I5" t="str">
-        <v>1. Navigate to User Management; 2. Click on Add User; 3. click on new internal user.; 4. enter first name.; 5. enter last name.; 6. Enter existing email address; 4. Click on Save</v>
+        <v>1. Navigate to User Management; 2. Click on Add User; 3. click on add internal user.; 4. enter first name.; 5. enter last name.; 6. Enter existing email address; 4. Click on Save</v>
       </c>
       <c r="J5" t="str">
         <v>1. User Management page is displayed.; 2. Add User form is displayed.; 3. Email field shows entered value.; 4. Error message displays: 'Email already exists.'; Overall: System prevents duplicate email from being registered.</v>

</xml_diff>

<commit_message>
feat: generate user management test cases and refactor core automation modules for improved selection and parsing logic
</commit_message>
<xml_diff>
--- a/input/UC_trail_pw.xlsx
+++ b/input/UC_trail_pw.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011" filterPrivacy="true"/>
   <sheets>
     <sheet name="in" sheetId="1" r:id="rId1"/>
   </sheets>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -537,7 +537,7 @@
         <v>['Role: Dropdown (must exist in Role Management)']</v>
       </c>
       <c r="I3" t="str">
-        <v>1. Navigate to User Management.; 2.Click on  search.; 3. search the user by name or email.; 4. Click on the User.; 5. select edit.; 6. Open role dropdown.; 7. Select the role.; 6. Click on Save.</v>
+        <v>1. Navigate to User Management.; 2.Click on search.; 3. search the user by name or email.; 4. Click on the User.; 5. select edit.; 6. Open role dropdown.; 7. Select the role.; 6. Click on Save.</v>
       </c>
       <c r="J3" t="str">
         <v>1. User Management page is displayed.; 2. User details are displayed.; 3. Role dropdown reflects the chosen role.; 4. User role is updated successfully.; Overall: User's assigned role reflects changes in the user list.</v>
@@ -679,9 +679,65 @@
         <v>Final</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC-UM-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Verify reactivation of a user</v>
+      </c>
+      <c r="C6" t="str">
+        <v>User Management</v>
+      </c>
+      <c r="D6" t="str">
+        <v>User Status Management</v>
+      </c>
+      <c r="E6" t="str">
+        <v>FSD ID FS-RL-CF-04: Reactivated users can access the platform.</v>
+      </c>
+      <c r="F6" t="str">
+        <v>To ensure a Client admin can reactivate a user.</v>
+      </c>
+      <c r="G6" t="str">
+        <v>1. User is deactivated and exists in the system.; 2. Administrator is logged in.</v>
+      </c>
+      <c r="H6" t="str">
+        <v>['Status: Dropdown (must change from Deactivated to Active)']</v>
+      </c>
+      <c r="I6" t="str">
+        <v>1. Navigate to User Management; 2. Click on search.; 3. search the user by name or email id.; 4. Click on the user.; 5. Click on Reactivate.; 6. enter the comment in add comments.; 7. click on reactivate.</v>
+      </c>
+      <c r="J6" t="str">
+        <v>1. User Management page is displayed.; 2. User details are displayed.; 3. User status is updated to Active.; Overall: User can sign in post-reactivation.</v>
+      </c>
+      <c r="K6" t="str">
+        <v>User status reflects Active.</v>
+      </c>
+      <c r="L6" t="str">
+        <v>User status remains Deactivated.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Functional - Positive</v>
+      </c>
+      <c r="N6" t="str">
+        <v>P1</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Functional suitability</v>
+      </c>
+      <c r="P6" t="str">
+        <v>High</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Final</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>